<commit_message>
change title for SOC2 2017 revision 2022 (#1353)
change title
</commit_message>
<xml_diff>
--- a/tools/aicpa/SOC2_2017_with_rev_2022.xlsx
+++ b/tools/aicpa/SOC2_2017_with_rev_2022.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericlaubacher/Documents/GitHub/ciso-assistant-community/tools/aicpa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49C2C304-3412-F846-8971-2220FF7A7628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C0636A7-AB61-9442-BA3D-3D4AFC5722EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="160" yWindow="500" windowWidth="34240" windowHeight="20580" xr2:uid="{D01D941C-8F4B-437A-8397-2B749EA54579}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1505" uniqueCount="1193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1505" uniqueCount="1194">
   <si>
     <t>System Operations</t>
   </si>
@@ -3673,6 +3673,9 @@
   </si>
   <si>
     <t>CC5</t>
+  </si>
+  <si>
+    <t>SOC2-2017 Trust Services Criteria (revision 2022)</t>
   </si>
 </sst>
 </file>
@@ -4255,7 +4258,7 @@
         <v>1144</v>
       </c>
       <c r="B5" s="31" t="s">
-        <v>1145</v>
+        <v>1193</v>
       </c>
       <c r="C5" s="31"/>
     </row>
@@ -4327,7 +4330,7 @@
         <v>1155</v>
       </c>
       <c r="B13" s="31" t="s">
-        <v>1145</v>
+        <v>1193</v>
       </c>
       <c r="C13" s="31"/>
     </row>

</xml_diff>